<commit_message>
📊 semana XX - sincronizado
</commit_message>
<xml_diff>
--- a/Tracking-Body-Sculp.xlsx
+++ b/Tracking-Body-Sculp.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="71">
   <si>
     <t>Fecha</t>
   </si>
@@ -55,6 +55,9 @@
     <t>Muñeca (cm)</t>
   </si>
   <si>
+    <t>Cuello (cm)</t>
+  </si>
+  <si>
     <t>Masa Muscular (kg)</t>
   </si>
   <si>
@@ -191,9 +194,6 @@
   </si>
   <si>
     <t>Medida Otros</t>
-  </si>
-  <si>
-    <t>Cuello (cm)</t>
   </si>
   <si>
     <t>42.1 cm</t>
@@ -267,7 +267,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -300,6 +300,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -570,6 +573,9 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="3">
@@ -611,6 +617,9 @@
       <c r="M2" s="1">
         <v>17.5</v>
       </c>
+      <c r="N2" s="1">
+        <v>41.0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3">
@@ -652,6 +661,9 @@
       <c r="M3" s="1">
         <v>17.5</v>
       </c>
+      <c r="N3" s="1">
+        <v>41.0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3">
@@ -692,6 +704,53 @@
       </c>
       <c r="M4" s="1">
         <v>17.5</v>
+      </c>
+      <c r="N4" s="1">
+        <v>41.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3">
+        <v>46088.0</v>
+      </c>
+      <c r="B5" s="1">
+        <v>88.56</v>
+      </c>
+      <c r="C5" s="1">
+        <v>22.62</v>
+      </c>
+      <c r="D5" s="1">
+        <v>24.79</v>
+      </c>
+      <c r="E5" s="1">
+        <v>93.0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>124.0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>112.0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>39.0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>31.0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>95.0</v>
+      </c>
+      <c r="K5" s="1">
+        <v>56.0</v>
+      </c>
+      <c r="L5" s="1">
+        <v>38.0</v>
+      </c>
+      <c r="M5" s="1">
+        <v>17.5</v>
+      </c>
+      <c r="N5" s="1">
+        <v>41.0</v>
       </c>
     </row>
   </sheetData>
@@ -711,22 +770,22 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2">
@@ -766,13 +825,13 @@
         <v>19.56</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -864,6 +923,29 @@
         <v>14.82</v>
       </c>
       <c r="G7" s="1">
+        <v>44.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3">
+        <v>46088.0</v>
+      </c>
+      <c r="B8" s="1">
+        <v>64.79</v>
+      </c>
+      <c r="C8" s="1">
+        <v>13.0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>18.27</v>
+      </c>
+      <c r="E8" s="1">
+        <v>56.48</v>
+      </c>
+      <c r="F8" s="1">
+        <v>14.77</v>
+      </c>
+      <c r="G8" s="1">
         <v>44.0</v>
       </c>
     </row>
@@ -881,220 +963,220 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C3" s="4">
         <v>23.0</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="9">
         <v>0.13</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="4">
         <v>5.0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" s="4">
         <v>1.618</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>59</v>
+        <v>13</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>60</v>
@@ -1181,7 +1263,7 @@
         <v>0.41</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4">
@@ -1227,7 +1309,7 @@
         <v>0.4</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -1273,7 +1355,7 @@
         <v>0.29</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -1297,6 +1379,29 @@
       </c>
       <c r="G8" s="2" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3">
+        <v>46088.0</v>
+      </c>
+      <c r="B9" s="1">
+        <v>1386.0</v>
+      </c>
+      <c r="C9" s="1">
+        <v>546.0</v>
+      </c>
+      <c r="D9" s="11">
+        <v>0.4</v>
+      </c>
+      <c r="E9" s="11">
+        <v>0.33</v>
+      </c>
+      <c r="F9" s="11">
+        <v>0.27</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>